<commit_message>
Add missing bus stands and private/govt bus routes to Excel directories
- Cross-checked both workbooks: every route terminal/via place vs the
  stands sheet, and both against published WBTC/private route lists
- Stands: 134 -> 193 (official WBTIDCL terminals + route termini)
- Routes: 160 -> 466 (missing WBTC, 200-series, DN/SD/KB, minibus,
  RT/M/MM/MN and blue-yellow private routes with published terminals
  and via stops; timetable/fleet/registrations left blank where not
  verifiable - no invented data)
- Fixed stale summary formulas and restored Master Index sheet links
- Added data/MISSING_DATA_AUDIT.md documenting additions, matched
  terminal variants, per-route fleet/registration gaps and number
  conflicts for transport office verification
- Excel only: website data file not regenerated

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/Kolkata_Bus_Stands_v2.xlsx
+++ b/data/Kolkata_Bus_Stands_v2.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -621,22 +621,22 @@
     </row>
     <row r="5">
       <c r="A5" s="5">
-        <f>COUNTA(A8:A87)</f>
+        <f>COUNTA(A8:A1000)</f>
         <v/>
       </c>
       <c r="B5" s="11" t="n"/>
       <c r="C5" s="5">
-        <f>COUNTIF(D8:D87, "*Depot*")</f>
+        <f>COUNTIF(D8:D1000, "*Depot*")</f>
         <v/>
       </c>
       <c r="D5" s="11" t="n"/>
       <c r="E5" s="5">
-        <f>COUNTIF(D8:D87, "*Terminal*")</f>
+        <f>COUNTIF(D8:D1000, "*Terminal*")</f>
         <v/>
       </c>
       <c r="F5" s="11" t="n"/>
       <c r="G5" s="5">
-        <f>COUNTIF(D8:D87, "*Stand*")</f>
+        <f>COUNTIF(D8:D1000, "*Stand*")</f>
         <v/>
       </c>
     </row>
@@ -4983,6 +4983,1635 @@
         </is>
       </c>
       <c r="G141" s="10" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="9" t="n">
+        <v>135</v>
+      </c>
+      <c r="B142" s="10" t="inlineStr">
+        <is>
+          <t>Bagnan Bus Terminus</t>
+        </is>
+      </c>
+      <c r="C142" s="10" t="inlineStr">
+        <is>
+          <t>Bagnan Stand</t>
+        </is>
+      </c>
+      <c r="D142" s="9" t="inlineStr">
+        <is>
+          <t>Major Passenger Terminal</t>
+        </is>
+      </c>
+      <c r="E142" s="10" t="inlineStr">
+        <is>
+          <t>WBTIDCL</t>
+        </is>
+      </c>
+      <c r="F142" s="10" t="inlineStr">
+        <is>
+          <t>Bagnan, Howrah</t>
+        </is>
+      </c>
+      <c r="G142" s="10" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="9" t="n">
+        <v>136</v>
+      </c>
+      <c r="B143" s="10" t="inlineStr">
+        <is>
+          <t>Uluberia Bus Terminus</t>
+        </is>
+      </c>
+      <c r="C143" s="10" t="inlineStr">
+        <is>
+          <t>Uluberia Stand</t>
+        </is>
+      </c>
+      <c r="D143" s="9" t="inlineStr">
+        <is>
+          <t>Major Passenger Terminal</t>
+        </is>
+      </c>
+      <c r="E143" s="10" t="inlineStr">
+        <is>
+          <t>WBTIDCL</t>
+        </is>
+      </c>
+      <c r="F143" s="10" t="inlineStr">
+        <is>
+          <t>Uluberia, Howrah</t>
+        </is>
+      </c>
+      <c r="G143" s="10" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="9" t="n">
+        <v>137</v>
+      </c>
+      <c r="B144" s="10" t="inlineStr">
+        <is>
+          <t>Udaynarayanpur Bus Terminus</t>
+        </is>
+      </c>
+      <c r="C144" s="10" t="inlineStr">
+        <is>
+          <t>Udaynarayanpur Stand</t>
+        </is>
+      </c>
+      <c r="D144" s="9" t="inlineStr">
+        <is>
+          <t>Major Passenger Terminal</t>
+        </is>
+      </c>
+      <c r="E144" s="10" t="inlineStr">
+        <is>
+          <t>WBTIDCL</t>
+        </is>
+      </c>
+      <c r="F144" s="10" t="inlineStr">
+        <is>
+          <t>Udaynarayanpur, Howrah</t>
+        </is>
+      </c>
+      <c r="G144" s="10" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="9" t="n">
+        <v>138</v>
+      </c>
+      <c r="B145" s="10" t="inlineStr">
+        <is>
+          <t>Gadiara Bus Terminus</t>
+        </is>
+      </c>
+      <c r="C145" s="10" t="inlineStr">
+        <is>
+          <t>Gadiara Stand</t>
+        </is>
+      </c>
+      <c r="D145" s="9" t="inlineStr">
+        <is>
+          <t>Major Passenger Terminal</t>
+        </is>
+      </c>
+      <c r="E145" s="10" t="inlineStr">
+        <is>
+          <t>WBTIDCL</t>
+        </is>
+      </c>
+      <c r="F145" s="10" t="inlineStr">
+        <is>
+          <t>Gadiara, Howrah</t>
+        </is>
+      </c>
+      <c r="G145" s="10" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="9" t="n">
+        <v>139</v>
+      </c>
+      <c r="B146" s="10" t="inlineStr">
+        <is>
+          <t>Raidighi Bus Terminus</t>
+        </is>
+      </c>
+      <c r="C146" s="10" t="inlineStr">
+        <is>
+          <t>Raidighi Stand</t>
+        </is>
+      </c>
+      <c r="D146" s="9" t="inlineStr">
+        <is>
+          <t>Major Passenger Terminal</t>
+        </is>
+      </c>
+      <c r="E146" s="10" t="inlineStr">
+        <is>
+          <t>WBTIDCL</t>
+        </is>
+      </c>
+      <c r="F146" s="10" t="inlineStr">
+        <is>
+          <t>Raidighi, South 24 Parganas</t>
+        </is>
+      </c>
+      <c r="G146" s="10" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="9" t="n">
+        <v>140</v>
+      </c>
+      <c r="B147" s="10" t="inlineStr">
+        <is>
+          <t>Usthi Bus Terminus</t>
+        </is>
+      </c>
+      <c r="C147" s="10" t="inlineStr">
+        <is>
+          <t>Usthi Stand</t>
+        </is>
+      </c>
+      <c r="D147" s="9" t="inlineStr">
+        <is>
+          <t>Major Passenger Terminal</t>
+        </is>
+      </c>
+      <c r="E147" s="10" t="inlineStr">
+        <is>
+          <t>WBTIDCL</t>
+        </is>
+      </c>
+      <c r="F147" s="10" t="inlineStr">
+        <is>
+          <t>Usthi, South 24 Parganas</t>
+        </is>
+      </c>
+      <c r="G147" s="10" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="9" t="n">
+        <v>141</v>
+      </c>
+      <c r="B148" s="10" t="inlineStr">
+        <is>
+          <t>Kakdwip Lot 8 Bus Terminus</t>
+        </is>
+      </c>
+      <c r="C148" s="10" t="inlineStr">
+        <is>
+          <t>Lot 8 Stand</t>
+        </is>
+      </c>
+      <c r="D148" s="9" t="inlineStr">
+        <is>
+          <t>Major Passenger Terminal</t>
+        </is>
+      </c>
+      <c r="E148" s="10" t="inlineStr">
+        <is>
+          <t>WBTIDCL</t>
+        </is>
+      </c>
+      <c r="F148" s="10" t="inlineStr">
+        <is>
+          <t>Kakdwip, South 24 Parganas</t>
+        </is>
+      </c>
+      <c r="G148" s="10" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="9" t="n">
+        <v>142</v>
+      </c>
+      <c r="B149" s="10" t="inlineStr">
+        <is>
+          <t>Diamond Harbour Bus Terminus</t>
+        </is>
+      </c>
+      <c r="C149" s="10" t="inlineStr">
+        <is>
+          <t>Diamond Harbour Stand</t>
+        </is>
+      </c>
+      <c r="D149" s="9" t="inlineStr">
+        <is>
+          <t>Major Passenger Terminal</t>
+        </is>
+      </c>
+      <c r="E149" s="10" t="inlineStr">
+        <is>
+          <t>WBTIDCL</t>
+        </is>
+      </c>
+      <c r="F149" s="10" t="inlineStr">
+        <is>
+          <t>Diamond Harbour, South 24 Parganas</t>
+        </is>
+      </c>
+      <c r="G149" s="10" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="9" t="n">
+        <v>143</v>
+      </c>
+      <c r="B150" s="10" t="inlineStr">
+        <is>
+          <t>Kachuberia Bus Terminus</t>
+        </is>
+      </c>
+      <c r="C150" s="10" t="inlineStr">
+        <is>
+          <t>Kachuberia Stand</t>
+        </is>
+      </c>
+      <c r="D150" s="9" t="inlineStr">
+        <is>
+          <t>Major Passenger Terminal</t>
+        </is>
+      </c>
+      <c r="E150" s="10" t="inlineStr">
+        <is>
+          <t>WBTIDCL</t>
+        </is>
+      </c>
+      <c r="F150" s="10" t="inlineStr">
+        <is>
+          <t>Kachuberia, Sagar Island, South 24 Parganas</t>
+        </is>
+      </c>
+      <c r="G150" s="10" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="9" t="n">
+        <v>144</v>
+      </c>
+      <c r="B151" s="10" t="inlineStr">
+        <is>
+          <t>Dum Dum Station Bus Stand</t>
+        </is>
+      </c>
+      <c r="C151" s="10" t="inlineStr">
+        <is>
+          <t>Dum Dum Station Stand</t>
+        </is>
+      </c>
+      <c r="D151" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E151" s="10" t="inlineStr">
+        <is>
+          <t>WBTC / Private Operators</t>
+        </is>
+      </c>
+      <c r="F151" s="10" t="n"/>
+      <c r="G151" s="10" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="9" t="n">
+        <v>145</v>
+      </c>
+      <c r="B152" s="10" t="inlineStr">
+        <is>
+          <t>Naihati Bus Terminus</t>
+        </is>
+      </c>
+      <c r="C152" s="10" t="inlineStr">
+        <is>
+          <t>Naihati Stand</t>
+        </is>
+      </c>
+      <c r="D152" s="9" t="inlineStr">
+        <is>
+          <t>Major Passenger Terminal</t>
+        </is>
+      </c>
+      <c r="E152" s="10" t="inlineStr">
+        <is>
+          <t>WBTC / Private Operators</t>
+        </is>
+      </c>
+      <c r="F152" s="10" t="n"/>
+      <c r="G152" s="10" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="9" t="n">
+        <v>146</v>
+      </c>
+      <c r="B153" s="10" t="inlineStr">
+        <is>
+          <t>Kankurgachi Bus Stand</t>
+        </is>
+      </c>
+      <c r="C153" s="10" t="inlineStr">
+        <is>
+          <t>Kankurgachi Stand</t>
+        </is>
+      </c>
+      <c r="D153" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E153" s="10" t="inlineStr">
+        <is>
+          <t>WBTC / Private Operators</t>
+        </is>
+      </c>
+      <c r="F153" s="10" t="n"/>
+      <c r="G153" s="10" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="9" t="n">
+        <v>147</v>
+      </c>
+      <c r="B154" s="10" t="inlineStr">
+        <is>
+          <t>Madhyamgram Bus Stand</t>
+        </is>
+      </c>
+      <c r="C154" s="10" t="inlineStr">
+        <is>
+          <t>Madhyamgram Chowmatha Stand</t>
+        </is>
+      </c>
+      <c r="D154" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E154" s="10" t="inlineStr">
+        <is>
+          <t>WBTC / Private Operators</t>
+        </is>
+      </c>
+      <c r="F154" s="10" t="n"/>
+      <c r="G154" s="10" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="9" t="n">
+        <v>148</v>
+      </c>
+      <c r="B155" s="10" t="inlineStr">
+        <is>
+          <t>Munshirhat Bus Stand</t>
+        </is>
+      </c>
+      <c r="C155" s="10" t="inlineStr">
+        <is>
+          <t>Munshirhat Stand</t>
+        </is>
+      </c>
+      <c r="D155" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E155" s="10" t="inlineStr">
+        <is>
+          <t>WBTC</t>
+        </is>
+      </c>
+      <c r="F155" s="10" t="n"/>
+      <c r="G155" s="10" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="9" t="n">
+        <v>149</v>
+      </c>
+      <c r="B156" s="10" t="inlineStr">
+        <is>
+          <t>Sankrail Bus Stand</t>
+        </is>
+      </c>
+      <c r="C156" s="10" t="inlineStr">
+        <is>
+          <t>Sankrail Stand</t>
+        </is>
+      </c>
+      <c r="D156" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E156" s="10" t="inlineStr">
+        <is>
+          <t>WBTC</t>
+        </is>
+      </c>
+      <c r="F156" s="10" t="n"/>
+      <c r="G156" s="10" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="B157" s="10" t="inlineStr">
+        <is>
+          <t>Domjur Bus Stand</t>
+        </is>
+      </c>
+      <c r="C157" s="10" t="inlineStr">
+        <is>
+          <t>Domjur Stand</t>
+        </is>
+      </c>
+      <c r="D157" s="9" t="inlineStr">
+        <is>
+          <t>Major Passenger Terminal</t>
+        </is>
+      </c>
+      <c r="E157" s="10" t="inlineStr">
+        <is>
+          <t>WBTC / Private Operators</t>
+        </is>
+      </c>
+      <c r="F157" s="10" t="n"/>
+      <c r="G157" s="10" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="9" t="n">
+        <v>151</v>
+      </c>
+      <c r="B158" s="10" t="inlineStr">
+        <is>
+          <t>Badartala Bus Stand</t>
+        </is>
+      </c>
+      <c r="C158" s="10" t="inlineStr">
+        <is>
+          <t>Badartala Stand</t>
+        </is>
+      </c>
+      <c r="D158" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E158" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F158" s="10" t="n"/>
+      <c r="G158" s="10" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="9" t="n">
+        <v>152</v>
+      </c>
+      <c r="B159" s="10" t="inlineStr">
+        <is>
+          <t>Barisha Bus Stand</t>
+        </is>
+      </c>
+      <c r="C159" s="10" t="inlineStr">
+        <is>
+          <t>Barisha Stand</t>
+        </is>
+      </c>
+      <c r="D159" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E159" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F159" s="10" t="n"/>
+      <c r="G159" s="10" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="9" t="n">
+        <v>153</v>
+      </c>
+      <c r="B160" s="10" t="inlineStr">
+        <is>
+          <t>Sinthee Bus Stand</t>
+        </is>
+      </c>
+      <c r="C160" s="10" t="inlineStr">
+        <is>
+          <t>Sinthee More Stand</t>
+        </is>
+      </c>
+      <c r="D160" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E160" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F160" s="10" t="n"/>
+      <c r="G160" s="10" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="9" t="n">
+        <v>154</v>
+      </c>
+      <c r="B161" s="10" t="inlineStr">
+        <is>
+          <t>Dhakuria Bus Stand</t>
+        </is>
+      </c>
+      <c r="C161" s="10" t="inlineStr">
+        <is>
+          <t>Dhakuria Stand</t>
+        </is>
+      </c>
+      <c r="D161" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E161" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F161" s="10" t="n"/>
+      <c r="G161" s="10" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="9" t="n">
+        <v>155</v>
+      </c>
+      <c r="B162" s="10" t="inlineStr">
+        <is>
+          <t>Picnic Garden Bus Stand</t>
+        </is>
+      </c>
+      <c r="C162" s="10" t="inlineStr">
+        <is>
+          <t>Picnic Garden Stand</t>
+        </is>
+      </c>
+      <c r="D162" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E162" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F162" s="10" t="n"/>
+      <c r="G162" s="10" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="9" t="n">
+        <v>156</v>
+      </c>
+      <c r="B163" s="10" t="inlineStr">
+        <is>
+          <t>Alampur Bus Stand</t>
+        </is>
+      </c>
+      <c r="C163" s="10" t="inlineStr">
+        <is>
+          <t>Alampur Stand</t>
+        </is>
+      </c>
+      <c r="D163" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E163" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F163" s="10" t="n"/>
+      <c r="G163" s="10" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="9" t="n">
+        <v>157</v>
+      </c>
+      <c r="B164" s="10" t="inlineStr">
+        <is>
+          <t>Dasnagar Bus Stand</t>
+        </is>
+      </c>
+      <c r="C164" s="10" t="inlineStr">
+        <is>
+          <t>Dasnagar Stand</t>
+        </is>
+      </c>
+      <c r="D164" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E164" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F164" s="10" t="n"/>
+      <c r="G164" s="10" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="9" t="n">
+        <v>158</v>
+      </c>
+      <c r="B165" s="10" t="inlineStr">
+        <is>
+          <t>Kadamtala Bus Stand</t>
+        </is>
+      </c>
+      <c r="C165" s="10" t="inlineStr">
+        <is>
+          <t>Kadamtala Stand</t>
+        </is>
+      </c>
+      <c r="D165" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E165" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F165" s="10" t="n"/>
+      <c r="G165" s="10" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="9" t="n">
+        <v>159</v>
+      </c>
+      <c r="B166" s="10" t="inlineStr">
+        <is>
+          <t>Kanchrapara Bus Stand</t>
+        </is>
+      </c>
+      <c r="C166" s="10" t="inlineStr">
+        <is>
+          <t>Kanchrapara Stand</t>
+        </is>
+      </c>
+      <c r="D166" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E166" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F166" s="10" t="n"/>
+      <c r="G166" s="10" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="9" t="n">
+        <v>160</v>
+      </c>
+      <c r="B167" s="10" t="inlineStr">
+        <is>
+          <t>Milk Colony Bus Stand</t>
+        </is>
+      </c>
+      <c r="C167" s="10" t="inlineStr">
+        <is>
+          <t>Milk Colony Stand</t>
+        </is>
+      </c>
+      <c r="D167" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E167" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F167" s="10" t="n"/>
+      <c r="G167" s="10" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="9" t="n">
+        <v>161</v>
+      </c>
+      <c r="B168" s="10" t="inlineStr">
+        <is>
+          <t>Anandapur Bus Stand</t>
+        </is>
+      </c>
+      <c r="C168" s="10" t="inlineStr">
+        <is>
+          <t>Anandapur Stand</t>
+        </is>
+      </c>
+      <c r="D168" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E168" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F168" s="10" t="n"/>
+      <c r="G168" s="10" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="9" t="n">
+        <v>162</v>
+      </c>
+      <c r="B169" s="10" t="inlineStr">
+        <is>
+          <t>Nagerbazar Bus Stand</t>
+        </is>
+      </c>
+      <c r="C169" s="10" t="inlineStr">
+        <is>
+          <t>Nagerbazar Stand</t>
+        </is>
+      </c>
+      <c r="D169" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E169" s="10" t="inlineStr">
+        <is>
+          <t>WBTC / Private Operators</t>
+        </is>
+      </c>
+      <c r="F169" s="10" t="n"/>
+      <c r="G169" s="10" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="9" t="n">
+        <v>163</v>
+      </c>
+      <c r="B170" s="10" t="inlineStr">
+        <is>
+          <t>Bongaon Bus Stand</t>
+        </is>
+      </c>
+      <c r="C170" s="10" t="inlineStr">
+        <is>
+          <t>Bongaon Stand</t>
+        </is>
+      </c>
+      <c r="D170" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E170" s="10" t="inlineStr">
+        <is>
+          <t>WBTC / Private Operators</t>
+        </is>
+      </c>
+      <c r="F170" s="10" t="n"/>
+      <c r="G170" s="10" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="9" t="n">
+        <v>164</v>
+      </c>
+      <c r="B171" s="10" t="inlineStr">
+        <is>
+          <t>Basirhat Bus Stand</t>
+        </is>
+      </c>
+      <c r="C171" s="10" t="inlineStr">
+        <is>
+          <t>Basirhat Stand</t>
+        </is>
+      </c>
+      <c r="D171" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E171" s="10" t="inlineStr">
+        <is>
+          <t>WBTC / Private Operators</t>
+        </is>
+      </c>
+      <c r="F171" s="10" t="n"/>
+      <c r="G171" s="10" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="9" t="n">
+        <v>165</v>
+      </c>
+      <c r="B172" s="10" t="inlineStr">
+        <is>
+          <t>Baduria Bus Stand</t>
+        </is>
+      </c>
+      <c r="C172" s="10" t="inlineStr">
+        <is>
+          <t>Baduria Stand</t>
+        </is>
+      </c>
+      <c r="D172" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E172" s="10" t="inlineStr">
+        <is>
+          <t>WBTC / Private Operators</t>
+        </is>
+      </c>
+      <c r="F172" s="10" t="n"/>
+      <c r="G172" s="10" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="9" t="n">
+        <v>166</v>
+      </c>
+      <c r="B173" s="10" t="inlineStr">
+        <is>
+          <t>Hasnabad Bus Stand</t>
+        </is>
+      </c>
+      <c r="C173" s="10" t="inlineStr">
+        <is>
+          <t>Hasnabad Stand</t>
+        </is>
+      </c>
+      <c r="D173" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E173" s="10" t="inlineStr">
+        <is>
+          <t>WBTC / Private Operators</t>
+        </is>
+      </c>
+      <c r="F173" s="10" t="n"/>
+      <c r="G173" s="10" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="9" t="n">
+        <v>167</v>
+      </c>
+      <c r="B174" s="10" t="inlineStr">
+        <is>
+          <t>Hakimpur Bus Stand</t>
+        </is>
+      </c>
+      <c r="C174" s="10" t="inlineStr">
+        <is>
+          <t>Hakimpur Stand</t>
+        </is>
+      </c>
+      <c r="D174" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E174" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F174" s="10" t="n"/>
+      <c r="G174" s="10" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="9" t="n">
+        <v>168</v>
+      </c>
+      <c r="B175" s="10" t="inlineStr">
+        <is>
+          <t>Dhamakhali Bus Stand</t>
+        </is>
+      </c>
+      <c r="C175" s="10" t="inlineStr">
+        <is>
+          <t>Dhamakhali Stand</t>
+        </is>
+      </c>
+      <c r="D175" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E175" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F175" s="10" t="n"/>
+      <c r="G175" s="10" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="9" t="n">
+        <v>169</v>
+      </c>
+      <c r="B176" s="10" t="inlineStr">
+        <is>
+          <t>Haroa Bus Stand</t>
+        </is>
+      </c>
+      <c r="C176" s="10" t="inlineStr">
+        <is>
+          <t>Haroa Stand</t>
+        </is>
+      </c>
+      <c r="D176" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E176" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F176" s="10" t="n"/>
+      <c r="G176" s="10" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="9" t="n">
+        <v>170</v>
+      </c>
+      <c r="B177" s="10" t="inlineStr">
+        <is>
+          <t>Ghatakpukur Bus Stand</t>
+        </is>
+      </c>
+      <c r="C177" s="10" t="inlineStr">
+        <is>
+          <t>Ghatakpukur Stand</t>
+        </is>
+      </c>
+      <c r="D177" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E177" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F177" s="10" t="n"/>
+      <c r="G177" s="10" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="9" t="n">
+        <v>171</v>
+      </c>
+      <c r="B178" s="10" t="inlineStr">
+        <is>
+          <t>Canning Bus Stand</t>
+        </is>
+      </c>
+      <c r="C178" s="10" t="inlineStr">
+        <is>
+          <t>Canning Stand</t>
+        </is>
+      </c>
+      <c r="D178" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E178" s="10" t="inlineStr">
+        <is>
+          <t>WBTC / Private Operators</t>
+        </is>
+      </c>
+      <c r="F178" s="10" t="n"/>
+      <c r="G178" s="10" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="9" t="n">
+        <v>172</v>
+      </c>
+      <c r="B179" s="10" t="inlineStr">
+        <is>
+          <t>Joynagar Bus Stand</t>
+        </is>
+      </c>
+      <c r="C179" s="10" t="inlineStr">
+        <is>
+          <t>Joynagar Stand</t>
+        </is>
+      </c>
+      <c r="D179" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E179" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F179" s="10" t="n"/>
+      <c r="G179" s="10" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="9" t="n">
+        <v>173</v>
+      </c>
+      <c r="B180" s="10" t="inlineStr">
+        <is>
+          <t>Sonarpur Bus Stand</t>
+        </is>
+      </c>
+      <c r="C180" s="10" t="inlineStr">
+        <is>
+          <t>Sonarpur Stand</t>
+        </is>
+      </c>
+      <c r="D180" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E180" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F180" s="10" t="n"/>
+      <c r="G180" s="10" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="9" t="n">
+        <v>174</v>
+      </c>
+      <c r="B181" s="10" t="inlineStr">
+        <is>
+          <t>Patharpratima Bus Stand</t>
+        </is>
+      </c>
+      <c r="C181" s="10" t="inlineStr">
+        <is>
+          <t>Patharpratima Stand</t>
+        </is>
+      </c>
+      <c r="D181" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E181" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F181" s="10" t="n"/>
+      <c r="G181" s="10" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="9" t="n">
+        <v>175</v>
+      </c>
+      <c r="B182" s="10" t="inlineStr">
+        <is>
+          <t>Noorpur Bus Stand</t>
+        </is>
+      </c>
+      <c r="C182" s="10" t="inlineStr">
+        <is>
+          <t>Noorpur Stand</t>
+        </is>
+      </c>
+      <c r="D182" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E182" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F182" s="10" t="n"/>
+      <c r="G182" s="10" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="9" t="n">
+        <v>176</v>
+      </c>
+      <c r="B183" s="10" t="inlineStr">
+        <is>
+          <t>Falta Bus Stand</t>
+        </is>
+      </c>
+      <c r="C183" s="10" t="inlineStr">
+        <is>
+          <t>Falta Stand</t>
+        </is>
+      </c>
+      <c r="D183" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E183" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F183" s="10" t="n"/>
+      <c r="G183" s="10" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="9" t="n">
+        <v>177</v>
+      </c>
+      <c r="B184" s="10" t="inlineStr">
+        <is>
+          <t>Amta Bus Stand</t>
+        </is>
+      </c>
+      <c r="C184" s="10" t="inlineStr">
+        <is>
+          <t>Amta Stand</t>
+        </is>
+      </c>
+      <c r="D184" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E184" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F184" s="10" t="n"/>
+      <c r="G184" s="10" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>178</v>
+      </c>
+      <c r="B185" s="10" t="inlineStr">
+        <is>
+          <t>Nimta Bus Stand</t>
+        </is>
+      </c>
+      <c r="C185" s="10" t="inlineStr">
+        <is>
+          <t>Nimta Stand</t>
+        </is>
+      </c>
+      <c r="D185" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E185" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F185" s="10" t="n"/>
+      <c r="G185" s="10" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="9" t="n">
+        <v>179</v>
+      </c>
+      <c r="B186" s="10" t="inlineStr">
+        <is>
+          <t>Belgharia Bus Stand</t>
+        </is>
+      </c>
+      <c r="C186" s="10" t="inlineStr">
+        <is>
+          <t>Belgharia Stand</t>
+        </is>
+      </c>
+      <c r="D186" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E186" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F186" s="10" t="n"/>
+      <c r="G186" s="10" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>180</v>
+      </c>
+      <c r="B187" s="10" t="inlineStr">
+        <is>
+          <t>Ahiritola Bus Stand</t>
+        </is>
+      </c>
+      <c r="C187" s="10" t="inlineStr">
+        <is>
+          <t>Ahiritola Stand</t>
+        </is>
+      </c>
+      <c r="D187" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E187" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F187" s="10" t="n"/>
+      <c r="G187" s="10" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="9" t="n">
+        <v>181</v>
+      </c>
+      <c r="B188" s="10" t="inlineStr">
+        <is>
+          <t>Kamarhati Bus Stand</t>
+        </is>
+      </c>
+      <c r="C188" s="10" t="inlineStr">
+        <is>
+          <t>Kamarhati Stand</t>
+        </is>
+      </c>
+      <c r="D188" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E188" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F188" s="10" t="n"/>
+      <c r="G188" s="10" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>182</v>
+      </c>
+      <c r="B189" s="10" t="inlineStr">
+        <is>
+          <t>Salkia Bus Stand</t>
+        </is>
+      </c>
+      <c r="C189" s="10" t="inlineStr">
+        <is>
+          <t>Salkia Stand</t>
+        </is>
+      </c>
+      <c r="D189" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E189" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F189" s="10" t="n"/>
+      <c r="G189" s="10" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="9" t="n">
+        <v>183</v>
+      </c>
+      <c r="B190" s="10" t="inlineStr">
+        <is>
+          <t>Chanditala Bus Stand</t>
+        </is>
+      </c>
+      <c r="C190" s="10" t="inlineStr">
+        <is>
+          <t>Chanditala Stand</t>
+        </is>
+      </c>
+      <c r="D190" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E190" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F190" s="10" t="n"/>
+      <c r="G190" s="10" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>184</v>
+      </c>
+      <c r="B191" s="10" t="inlineStr">
+        <is>
+          <t>Raichak Bus Stand</t>
+        </is>
+      </c>
+      <c r="C191" s="10" t="inlineStr">
+        <is>
+          <t>Raichak Stand</t>
+        </is>
+      </c>
+      <c r="D191" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E191" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F191" s="10" t="n"/>
+      <c r="G191" s="10" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="9" t="n">
+        <v>185</v>
+      </c>
+      <c r="B192" s="10" t="inlineStr">
+        <is>
+          <t>Gaighata Bus Stand</t>
+        </is>
+      </c>
+      <c r="C192" s="10" t="inlineStr">
+        <is>
+          <t>Gaighata Stand</t>
+        </is>
+      </c>
+      <c r="D192" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E192" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F192" s="10" t="n"/>
+      <c r="G192" s="10" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="n">
+        <v>186</v>
+      </c>
+      <c r="B193" s="10" t="inlineStr">
+        <is>
+          <t>Duttapukur Bus Stand</t>
+        </is>
+      </c>
+      <c r="C193" s="10" t="inlineStr">
+        <is>
+          <t>Duttapukur Stand</t>
+        </is>
+      </c>
+      <c r="D193" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E193" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F193" s="10" t="n"/>
+      <c r="G193" s="10" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="9" t="n">
+        <v>187</v>
+      </c>
+      <c r="B194" s="10" t="inlineStr">
+        <is>
+          <t>Hatishala Bus Stand</t>
+        </is>
+      </c>
+      <c r="C194" s="10" t="inlineStr">
+        <is>
+          <t>Hatishala Stand</t>
+        </is>
+      </c>
+      <c r="D194" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E194" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F194" s="10" t="n"/>
+      <c r="G194" s="10" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="B195" s="10" t="inlineStr">
+        <is>
+          <t>Ganganagar Bus Stand</t>
+        </is>
+      </c>
+      <c r="C195" s="10" t="inlineStr">
+        <is>
+          <t>Ganganagar Stand</t>
+        </is>
+      </c>
+      <c r="D195" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E195" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F195" s="10" t="n"/>
+      <c r="G195" s="10" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="B196" s="10" t="inlineStr">
+        <is>
+          <t>Birati Bus Stand</t>
+        </is>
+      </c>
+      <c r="C196" s="10" t="inlineStr">
+        <is>
+          <t>Birati Stand</t>
+        </is>
+      </c>
+      <c r="D196" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E196" s="10" t="inlineStr">
+        <is>
+          <t>WBTC / Private Operators</t>
+        </is>
+      </c>
+      <c r="F196" s="10" t="n"/>
+      <c r="G196" s="10" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="B197" s="10" t="inlineStr">
+        <is>
+          <t>Nahata Bus Stand</t>
+        </is>
+      </c>
+      <c r="C197" s="10" t="inlineStr">
+        <is>
+          <t>Nahata Stand</t>
+        </is>
+      </c>
+      <c r="D197" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E197" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F197" s="10" t="n"/>
+      <c r="G197" s="10" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="9" t="n">
+        <v>191</v>
+      </c>
+      <c r="B198" s="10" t="inlineStr">
+        <is>
+          <t>New Barrackpore Bus Stand</t>
+        </is>
+      </c>
+      <c r="C198" s="10" t="inlineStr">
+        <is>
+          <t>New Barrackpore Stand</t>
+        </is>
+      </c>
+      <c r="D198" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E198" s="10" t="inlineStr">
+        <is>
+          <t>WBTC / Private Operators</t>
+        </is>
+      </c>
+      <c r="F198" s="10" t="n"/>
+      <c r="G198" s="10" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="n">
+        <v>192</v>
+      </c>
+      <c r="B199" s="10" t="inlineStr">
+        <is>
+          <t>Rajchandrapur Bus Stand</t>
+        </is>
+      </c>
+      <c r="C199" s="10" t="inlineStr">
+        <is>
+          <t>Rajchandrapur Stand</t>
+        </is>
+      </c>
+      <c r="D199" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E199" s="10" t="inlineStr">
+        <is>
+          <t>WBTC / Private Operators</t>
+        </is>
+      </c>
+      <c r="F199" s="10" t="n"/>
+      <c r="G199" s="10" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="9" t="n">
+        <v>193</v>
+      </c>
+      <c r="B200" s="10" t="inlineStr">
+        <is>
+          <t>Kona Bus Stand</t>
+        </is>
+      </c>
+      <c r="C200" s="10" t="inlineStr">
+        <is>
+          <t>Kona More Stand</t>
+        </is>
+      </c>
+      <c r="D200" s="9" t="inlineStr">
+        <is>
+          <t>Route Stand &amp; Transit Node</t>
+        </is>
+      </c>
+      <c r="E200" s="10" t="inlineStr">
+        <is>
+          <t>Private Operators Syndicate</t>
+        </is>
+      </c>
+      <c r="F200" s="10" t="n"/>
+      <c r="G200" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
Revert "Stop publishing invented times and unconfirmed routes"
</commit_message>
<xml_diff>
--- a/data/Kolkata_Bus_Stands_v2.xlsx
+++ b/data/Kolkata_Bus_Stands_v2.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I200"/>
+  <dimension ref="A1:G200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -677,16 +677,6 @@
           <t>Key Functional Role &amp; Facilities</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Verification Note</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -722,16 +712,6 @@
           <t>Central Workshop, Fleet Maintenance, HQ Administration</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n">
@@ -767,16 +747,6 @@
           <t>Southern Suburban Route Anchor &amp; Fleet Parking Yard</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -812,16 +782,6 @@
           <t>Rail-Bus Multi-Modal Interchange Maintenance Hub</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n">
@@ -857,16 +817,6 @@
           <t>Eastern Bypass Operations &amp; Inter-District Fleet Yard</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -902,16 +852,6 @@
           <t>South-Central Intra-City Bus Terminal &amp; Yard</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n">
@@ -947,16 +887,6 @@
           <t>North-Central Arterial Maintenance Depot</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -992,16 +922,6 @@
           <t>Northern Suburban Boundary Anchor &amp; Long-Route Yard</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n">
@@ -1037,16 +957,6 @@
           <t>North Kolkata Fleet Maintenance &amp; Route Terminal</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -1082,16 +992,6 @@
           <t>IT Corridor &amp; Planned Township Operations Base</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="n">
@@ -1127,16 +1027,6 @@
           <t>Port &amp; South-Western Corridor Maintenance Base</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -1172,16 +1062,6 @@
           <t>Far-South Commuter Corridor Terminus &amp; Fleet Base</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="n">
@@ -1217,16 +1097,6 @@
           <t>Metro-Connected South Depot &amp; Tram-Bus Maintenance</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -1262,16 +1132,6 @@
           <t>Docklands &amp; West Kolkata Intra-City Yard</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="n">
@@ -1307,16 +1167,6 @@
           <t>High-Density South Corridor Intermediate Depot</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -1352,16 +1202,6 @@
           <t>South Kolkata Commercial Hub Maintenance Yard</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="n">
@@ -1397,16 +1237,6 @@
           <t>Central-East Arterial Intersection Depot</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -1442,16 +1272,6 @@
           <t>Central Rail Connector (Sealdah Corridor) Base</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n">
@@ -1487,16 +1307,6 @@
           <t>North-East Airport &amp; Bypass Transit Hub Base</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
@@ -1532,16 +1342,6 @@
           <t>North Metro Terminus &amp; Bus Maintenance Hub</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n">
@@ -1577,16 +1377,6 @@
           <t>Suburban District Boundary Depot &amp; Long-Distance Hub</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -1622,16 +1412,6 @@
           <t>Far North-East District Boundary Operations Base</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
@@ -1667,16 +1447,6 @@
           <t>South-Western Urban Fringe Fleet Yard &amp; Depot</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
@@ -1712,16 +1482,6 @@
           <t>Specialized IT Corridor &amp; Express Bus Depot</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n">
@@ -1757,16 +1517,6 @@
           <t>Smart City Satellite Depot &amp; Fleet Terminal</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
@@ -1802,16 +1552,6 @@
           <t>Modern Peripheral Mega-Housing Corridor Base</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="n">
@@ -1847,16 +1587,6 @@
           <t>South Bengal State Transport Kolkata Operational Base</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
@@ -1892,16 +1622,6 @@
           <t>North Bengal State Transport Express Fleet Depot</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="n">
@@ -1937,16 +1657,6 @@
           <t>Howrah Inner-City Tram-Bus Fleet Depot</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
@@ -1982,16 +1692,6 @@
           <t>Central Business District Intra-City &amp; Inter-State Hub</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="n">
@@ -2027,16 +1727,6 @@
           <t>Long-Distance Interstate &amp; Inter-District Terminal</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n">
@@ -2072,16 +1762,6 @@
           <t>Multi-Modal Rail-Ferry-Bus Commuter Terminal</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="n">
@@ -2117,16 +1797,6 @@
           <t>Satellite City Inter-State &amp; Express Bus Terminal</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n">
@@ -2162,16 +1832,6 @@
           <t>Planned Township &amp; IT Hub Central Transit Stand</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="n">
@@ -2207,16 +1867,6 @@
           <t>Educational Corridor &amp; South City Transit Terminal</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n">
@@ -2252,16 +1902,6 @@
           <t>High-Density Commuter Corridor Stand</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="n">
@@ -2297,16 +1937,6 @@
           <t>Outer Bypass Hub for South-Bound Inter-District Buses</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
@@ -2342,16 +1972,6 @@
           <t>Metro Feeder &amp; Southern Commuter Terminal</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="n">
@@ -2387,16 +2007,6 @@
           <t>Intermediate South-West Network Hub</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n">
@@ -2432,16 +2042,6 @@
           <t>Railway Feeder &amp; Port Industrial Passenger Hub</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="n">
@@ -2477,16 +2077,6 @@
           <t>Suburban Arterial Passenger Terminal</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n">
@@ -2522,16 +2112,6 @@
           <t>Riverfront Commuter &amp; Educational Zone Terminal</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="n">
@@ -2567,16 +2147,6 @@
           <t>Urban Sub-Terminal &amp; Commuter Hub</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="n">
@@ -2612,16 +2182,6 @@
           <t>Flyover Toll Interchange &amp; Inter-District Terminal</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="n">
@@ -2657,16 +2217,6 @@
           <t>Northern Gateway Inter-District Commuter Stand</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n">
@@ -2702,16 +2252,6 @@
           <t>Airport Corridor Arterial Passenger Terminal</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" s="9" t="n">
@@ -2747,16 +2287,6 @@
           <t>Suburban Rail-Bus Commuter Terminal</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n">
@@ -2792,16 +2322,6 @@
           <t>Pilgrimage &amp; Metro-Rail Multi-Modal Terminal</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n">
@@ -2837,16 +2357,6 @@
           <t>Highway Feeder &amp; Industrial Zone Terminal</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n">
@@ -2882,16 +2392,6 @@
           <t>Far-South Urban Commuter Gateway Stand</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" s="9" t="n">
@@ -2927,16 +2427,6 @@
           <t>High-Density Residential Colony Terminal</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n">
@@ -2972,16 +2462,6 @@
           <t>Industrial &amp; Residential Waterfront Passenger Hub</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59" s="9" t="n">
@@ -3017,16 +2497,6 @@
           <t>South 24 Parganas District HQ Commuter Terminal</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="n">
@@ -3062,16 +2532,6 @@
           <t>Long-Distance Express Train Feeder Terminal</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n">
@@ -3107,16 +2567,6 @@
           <t>South Kolkata Residential Colony Terminus</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="n">
@@ -3152,16 +2602,6 @@
           <t>Eastern Bypass Suburban Residential Terminal</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" s="9" t="n">
@@ -3197,16 +2637,6 @@
           <t>North Kolkata Primary Commercial Traffic Interchange</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="n">
@@ -3242,16 +2672,6 @@
           <t>Northern Gateway Arterial Interchange Hub</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" s="9" t="n">
@@ -3287,16 +2707,6 @@
           <t>South Kolkata Commercial Transit Node</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="n">
@@ -3332,16 +2742,6 @@
           <t>South-Central Traffic Intersection Stand</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" s="9" t="n">
@@ -3377,16 +2777,6 @@
           <t>Financial District Passenger Interchange</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="n">
@@ -3422,16 +2812,6 @@
           <t>Rail-Bus Major Commuter Interchange Node</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" s="9" t="n">
@@ -3467,16 +2847,6 @@
           <t>Airport Terminal Passenger Bus Interchange</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="n">
@@ -3512,16 +2882,6 @@
           <t>North-East Gateway Traffic Node</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" s="9" t="n">
@@ -3557,16 +2917,6 @@
           <t>IT Hub Commuter Transit Stand</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="72">
       <c r="A72" s="7" t="n">
@@ -3602,16 +2952,6 @@
           <t>Suburban South Colony Passenger Stand</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" s="9" t="n">
@@ -3647,16 +2987,6 @@
           <t>Southern Suburban Corridor Junction Stand</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="74">
       <c r="A74" s="7" t="n">
@@ -3692,16 +3022,6 @@
           <t>South-West Suburban Residential Terminus</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="75">
       <c r="A75" s="9" t="n">
@@ -3737,16 +3057,6 @@
           <t>South Suburban Residential Feeder Stand</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="76">
       <c r="A76" s="7" t="n">
@@ -3782,16 +3092,6 @@
           <t>North Suburban Riverfront Feeder Stand</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="77">
       <c r="A77" s="9" t="n">
@@ -3827,16 +3127,6 @@
           <t>Heritage Tram-Ferry-Bus Interchange Node</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="78">
       <c r="A78" s="7" t="n">
@@ -3872,16 +3162,6 @@
           <t>Far-West Behala Residential Colony Stand</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="79">
       <c r="A79" s="9" t="n">
@@ -3917,16 +3197,6 @@
           <t>Budge Budge Corridor Passenger Stand</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="80">
       <c r="A80" s="7" t="n">
@@ -3962,16 +3232,6 @@
           <t>Docklands &amp; Metiabruz Industrial Stand</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="81">
       <c r="A81" s="9" t="n">
@@ -4007,16 +3267,6 @@
           <t>Waterfront Super-Speciality Hospital Bus Hub</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="82">
       <c r="A82" s="7" t="n">
@@ -4052,16 +3302,6 @@
           <t>South Suburban Highway Transit Interchange</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="83">
       <c r="A83" s="9" t="n">
@@ -4097,16 +3337,6 @@
           <t>Industrial Corridor &amp; Durgapur Expressway Node</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="84">
       <c r="A84" s="7" t="n">
@@ -4142,16 +3372,6 @@
           <t>Central Corridor Arterial Transit Stand</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="85">
       <c r="A85" s="9" t="n">
@@ -4187,16 +3407,6 @@
           <t>Eastern Bypass Major Traffic Node</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="86">
       <c r="A86" s="7" t="n">
@@ -4232,16 +3442,6 @@
           <t>Medical &amp; Financial Hub Interchange Stand</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="87">
       <c r="A87" s="9" t="n">
@@ -4277,16 +3477,6 @@
           <t>Eastern Gateway Transit Interchange Node</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="88">
       <c r="A88" s="9" t="n">
@@ -4322,16 +3512,6 @@
           <t>Multi-storey southern terminus; AC, S-series and private routes; ticket counter, waiting room</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" s="9" t="n">
@@ -4367,16 +3547,6 @@
           <t>District bus terminal with 4 platforms; north-suburban and inter-district services</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>address and role from a published depot/terminal list</t>
-        </is>
-      </c>
     </row>
     <row r="90">
       <c r="A90" s="9" t="n">
@@ -4408,16 +3578,6 @@
         </is>
       </c>
       <c r="G90" s="10" t="n"/>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="91">
       <c r="A91" s="9" t="n">
@@ -4449,16 +3609,6 @@
         </is>
       </c>
       <c r="G91" s="10" t="n"/>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="92">
       <c r="A92" s="9" t="n">
@@ -4490,16 +3640,6 @@
         </is>
       </c>
       <c r="G92" s="10" t="n"/>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="93">
       <c r="A93" s="9" t="n">
@@ -4531,16 +3671,6 @@
         </is>
       </c>
       <c r="G93" s="10" t="n"/>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" s="9" t="n">
@@ -4572,16 +3702,6 @@
         </is>
       </c>
       <c r="G94" s="10" t="n"/>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="95">
       <c r="A95" s="9" t="n">
@@ -4613,16 +3733,6 @@
         </is>
       </c>
       <c r="G95" s="10" t="n"/>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="A96" s="9" t="n">
@@ -4650,16 +3760,6 @@
       </c>
       <c r="F96" s="10" t="n"/>
       <c r="G96" s="10" t="n"/>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="97">
       <c r="A97" s="9" t="n">
@@ -4687,16 +3787,6 @@
       </c>
       <c r="F97" s="10" t="n"/>
       <c r="G97" s="10" t="n"/>
-      <c r="H97" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I97" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="98">
       <c r="A98" s="9" t="n">
@@ -4724,16 +3814,6 @@
       </c>
       <c r="F98" s="10" t="n"/>
       <c r="G98" s="10" t="n"/>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I98" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="99">
       <c r="A99" s="9" t="n">
@@ -4761,16 +3841,6 @@
       </c>
       <c r="F99" s="10" t="n"/>
       <c r="G99" s="10" t="n"/>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="100">
       <c r="A100" s="9" t="n">
@@ -4798,16 +3868,6 @@
       </c>
       <c r="F100" s="10" t="n"/>
       <c r="G100" s="10" t="n"/>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="101">
       <c r="A101" s="9" t="n">
@@ -4835,16 +3895,6 @@
       </c>
       <c r="F101" s="10" t="n"/>
       <c r="G101" s="10" t="n"/>
-      <c r="H101" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="102">
       <c r="A102" s="9" t="n">
@@ -4872,16 +3922,6 @@
       </c>
       <c r="F102" s="10" t="n"/>
       <c r="G102" s="10" t="n"/>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="103">
       <c r="A103" s="9" t="n">
@@ -4909,16 +3949,6 @@
       </c>
       <c r="F103" s="10" t="n"/>
       <c r="G103" s="10" t="n"/>
-      <c r="H103" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I103" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="104">
       <c r="A104" s="9" t="n">
@@ -4946,16 +3976,6 @@
       </c>
       <c r="F104" s="10" t="n"/>
       <c r="G104" s="10" t="n"/>
-      <c r="H104" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="105">
       <c r="A105" s="9" t="n">
@@ -4983,16 +4003,6 @@
       </c>
       <c r="F105" s="10" t="n"/>
       <c r="G105" s="10" t="n"/>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="106">
       <c r="A106" s="9" t="n">
@@ -5020,16 +4030,6 @@
       </c>
       <c r="F106" s="10" t="n"/>
       <c r="G106" s="10" t="n"/>
-      <c r="H106" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I106" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="107">
       <c r="A107" s="9" t="n">
@@ -5057,16 +4057,6 @@
       </c>
       <c r="F107" s="10" t="n"/>
       <c r="G107" s="10" t="n"/>
-      <c r="H107" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I107" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="108">
       <c r="A108" s="9" t="n">
@@ -5094,16 +4084,6 @@
       </c>
       <c r="F108" s="10" t="n"/>
       <c r="G108" s="10" t="n"/>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="109">
       <c r="A109" s="9" t="n">
@@ -5131,16 +4111,6 @@
       </c>
       <c r="F109" s="10" t="n"/>
       <c r="G109" s="10" t="n"/>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="110">
       <c r="A110" s="9" t="n">
@@ -5168,16 +4138,6 @@
       </c>
       <c r="F110" s="10" t="n"/>
       <c r="G110" s="10" t="n"/>
-      <c r="H110" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="111">
       <c r="A111" s="9" t="n">
@@ -5205,16 +4165,6 @@
       </c>
       <c r="F111" s="10" t="n"/>
       <c r="G111" s="10" t="n"/>
-      <c r="H111" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="112">
       <c r="A112" s="9" t="n">
@@ -5242,16 +4192,6 @@
       </c>
       <c r="F112" s="10" t="n"/>
       <c r="G112" s="10" t="n"/>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="113">
       <c r="A113" s="9" t="n">
@@ -5279,16 +4219,6 @@
       </c>
       <c r="F113" s="10" t="n"/>
       <c r="G113" s="10" t="n"/>
-      <c r="H113" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="114">
       <c r="A114" s="9" t="n">
@@ -5316,16 +4246,6 @@
       </c>
       <c r="F114" s="10" t="n"/>
       <c r="G114" s="10" t="n"/>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I114" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="n">
@@ -5353,16 +4273,6 @@
       </c>
       <c r="F115" s="10" t="n"/>
       <c r="G115" s="10" t="n"/>
-      <c r="H115" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I115" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="116">
       <c r="A116" s="9" t="n">
@@ -5390,16 +4300,6 @@
       </c>
       <c r="F116" s="10" t="n"/>
       <c r="G116" s="10" t="n"/>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I116" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="117">
       <c r="A117" s="9" t="n">
@@ -5427,16 +4327,6 @@
       </c>
       <c r="F117" s="10" t="n"/>
       <c r="G117" s="10" t="n"/>
-      <c r="H117" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I117" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="118">
       <c r="A118" s="9" t="n">
@@ -5464,16 +4354,6 @@
       </c>
       <c r="F118" s="10" t="n"/>
       <c r="G118" s="10" t="n"/>
-      <c r="H118" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I118" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="119">
       <c r="A119" s="9" t="n">
@@ -5501,16 +4381,6 @@
       </c>
       <c r="F119" s="10" t="n"/>
       <c r="G119" s="10" t="n"/>
-      <c r="H119" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I119" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="120">
       <c r="A120" s="9" t="n">
@@ -5538,16 +4408,6 @@
       </c>
       <c r="F120" s="10" t="n"/>
       <c r="G120" s="10" t="n"/>
-      <c r="H120" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I120" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="121">
       <c r="A121" s="9" t="n">
@@ -5575,16 +4435,6 @@
       </c>
       <c r="F121" s="10" t="n"/>
       <c r="G121" s="10" t="n"/>
-      <c r="H121" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I121" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="122">
       <c r="A122" s="9" t="n">
@@ -5612,16 +4462,6 @@
       </c>
       <c r="F122" s="10" t="n"/>
       <c r="G122" s="10" t="n"/>
-      <c r="H122" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I122" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="123">
       <c r="A123" s="9" t="n">
@@ -5649,16 +4489,6 @@
       </c>
       <c r="F123" s="10" t="n"/>
       <c r="G123" s="10" t="n"/>
-      <c r="H123" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I123" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="124">
       <c r="A124" s="9" t="n">
@@ -5686,16 +4516,6 @@
       </c>
       <c r="F124" s="10" t="n"/>
       <c r="G124" s="10" t="n"/>
-      <c r="H124" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I124" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="125">
       <c r="A125" s="9" t="n">
@@ -5723,16 +4543,6 @@
       </c>
       <c r="F125" s="10" t="n"/>
       <c r="G125" s="10" t="n"/>
-      <c r="H125" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="126">
       <c r="A126" s="9" t="n">
@@ -5760,16 +4570,6 @@
       </c>
       <c r="F126" s="10" t="n"/>
       <c r="G126" s="10" t="n"/>
-      <c r="H126" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="127">
       <c r="A127" s="9" t="n">
@@ -5797,16 +4597,6 @@
       </c>
       <c r="F127" s="10" t="n"/>
       <c r="G127" s="10" t="n"/>
-      <c r="H127" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="128">
       <c r="A128" s="9" t="n">
@@ -5834,16 +4624,6 @@
       </c>
       <c r="F128" s="10" t="n"/>
       <c r="G128" s="10" t="n"/>
-      <c r="H128" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="129">
       <c r="A129" s="9" t="n">
@@ -5871,16 +4651,6 @@
       </c>
       <c r="F129" s="10" t="n"/>
       <c r="G129" s="10" t="n"/>
-      <c r="H129" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="130">
       <c r="A130" s="9" t="n">
@@ -5908,16 +4678,6 @@
       </c>
       <c r="F130" s="10" t="n"/>
       <c r="G130" s="10" t="n"/>
-      <c r="H130" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="131">
       <c r="A131" s="9" t="n">
@@ -5945,16 +4705,6 @@
       </c>
       <c r="F131" s="10" t="n"/>
       <c r="G131" s="10" t="n"/>
-      <c r="H131" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I131" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="132">
       <c r="A132" s="9" t="n">
@@ -5982,16 +4732,6 @@
       </c>
       <c r="F132" s="10" t="n"/>
       <c r="G132" s="10" t="n"/>
-      <c r="H132" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I132" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="133">
       <c r="A133" s="9" t="n">
@@ -6019,16 +4759,6 @@
       </c>
       <c r="F133" s="10" t="n"/>
       <c r="G133" s="10" t="n"/>
-      <c r="H133" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I133" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="134">
       <c r="A134" s="9" t="n">
@@ -6056,16 +4786,6 @@
       </c>
       <c r="F134" s="10" t="n"/>
       <c r="G134" s="10" t="n"/>
-      <c r="H134" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I134" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="135">
       <c r="A135" s="9" t="n">
@@ -6093,16 +4813,6 @@
       </c>
       <c r="F135" s="10" t="n"/>
       <c r="G135" s="10" t="n"/>
-      <c r="H135" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I135" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="136">
       <c r="A136" s="9" t="n">
@@ -6130,16 +4840,6 @@
       </c>
       <c r="F136" s="10" t="n"/>
       <c r="G136" s="10" t="n"/>
-      <c r="H136" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I136" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="137">
       <c r="A137" s="9" t="n">
@@ -6167,16 +4867,6 @@
       </c>
       <c r="F137" s="10" t="n"/>
       <c r="G137" s="10" t="n"/>
-      <c r="H137" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I137" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="138">
       <c r="A138" s="9" t="n">
@@ -6204,16 +4894,6 @@
       </c>
       <c r="F138" s="10" t="n"/>
       <c r="G138" s="10" t="n"/>
-      <c r="H138" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I138" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="139">
       <c r="A139" s="9" t="n">
@@ -6241,16 +4921,6 @@
       </c>
       <c r="F139" s="10" t="n"/>
       <c r="G139" s="10" t="n"/>
-      <c r="H139" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I139" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="140">
       <c r="A140" s="9" t="n">
@@ -6282,16 +4952,6 @@
         </is>
       </c>
       <c r="G140" s="10" t="n"/>
-      <c r="H140" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I140" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="141">
       <c r="A141" s="9" t="n">
@@ -6323,16 +4983,6 @@
         </is>
       </c>
       <c r="G141" s="10" t="n"/>
-      <c r="H141" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I141" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="142">
       <c r="A142" s="9" t="n">
@@ -6364,16 +5014,6 @@
         </is>
       </c>
       <c r="G142" s="10" t="n"/>
-      <c r="H142" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I142" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="143">
       <c r="A143" s="9" t="n">
@@ -6405,16 +5045,6 @@
         </is>
       </c>
       <c r="G143" s="10" t="n"/>
-      <c r="H143" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I143" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="144">
       <c r="A144" s="9" t="n">
@@ -6446,16 +5076,6 @@
         </is>
       </c>
       <c r="G144" s="10" t="n"/>
-      <c r="H144" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I144" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="145">
       <c r="A145" s="9" t="n">
@@ -6487,16 +5107,6 @@
         </is>
       </c>
       <c r="G145" s="10" t="n"/>
-      <c r="H145" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I145" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="146">
       <c r="A146" s="9" t="n">
@@ -6528,16 +5138,6 @@
         </is>
       </c>
       <c r="G146" s="10" t="n"/>
-      <c r="H146" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I146" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="147">
       <c r="A147" s="9" t="n">
@@ -6569,16 +5169,6 @@
         </is>
       </c>
       <c r="G147" s="10" t="n"/>
-      <c r="H147" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I147" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="148">
       <c r="A148" s="9" t="n">
@@ -6610,16 +5200,6 @@
         </is>
       </c>
       <c r="G148" s="10" t="n"/>
-      <c r="H148" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I148" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="149">
       <c r="A149" s="9" t="n">
@@ -6651,16 +5231,6 @@
         </is>
       </c>
       <c r="G149" s="10" t="n"/>
-      <c r="H149" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I149" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="150">
       <c r="A150" s="9" t="n">
@@ -6692,16 +5262,6 @@
         </is>
       </c>
       <c r="G150" s="10" t="n"/>
-      <c r="H150" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I150" t="inlineStr">
-        <is>
-          <t>no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="151">
       <c r="A151" s="9" t="n">
@@ -6729,16 +5289,6 @@
       </c>
       <c r="F151" s="10" t="n"/>
       <c r="G151" s="10" t="n"/>
-      <c r="H151" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I151" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="152">
       <c r="A152" s="9" t="n">
@@ -6766,16 +5316,6 @@
       </c>
       <c r="F152" s="10" t="n"/>
       <c r="G152" s="10" t="n"/>
-      <c r="H152" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I152" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="153">
       <c r="A153" s="9" t="n">
@@ -6803,16 +5343,6 @@
       </c>
       <c r="F153" s="10" t="n"/>
       <c r="G153" s="10" t="n"/>
-      <c r="H153" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="154">
       <c r="A154" s="9" t="n">
@@ -6840,16 +5370,6 @@
       </c>
       <c r="F154" s="10" t="n"/>
       <c r="G154" s="10" t="n"/>
-      <c r="H154" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I154" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="155">
       <c r="A155" s="9" t="n">
@@ -6877,16 +5397,6 @@
       </c>
       <c r="F155" s="10" t="n"/>
       <c r="G155" s="10" t="n"/>
-      <c r="H155" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I155" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="156">
       <c r="A156" s="9" t="n">
@@ -6914,16 +5424,6 @@
       </c>
       <c r="F156" s="10" t="n"/>
       <c r="G156" s="10" t="n"/>
-      <c r="H156" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I156" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="157">
       <c r="A157" s="9" t="n">
@@ -6951,16 +5451,6 @@
       </c>
       <c r="F157" s="10" t="n"/>
       <c r="G157" s="10" t="n"/>
-      <c r="H157" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I157" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="A158" s="9" t="n">
@@ -6988,16 +5478,6 @@
       </c>
       <c r="F158" s="10" t="n"/>
       <c r="G158" s="10" t="n"/>
-      <c r="H158" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I158" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="159">
       <c r="A159" s="9" t="n">
@@ -7025,16 +5505,6 @@
       </c>
       <c r="F159" s="10" t="n"/>
       <c r="G159" s="10" t="n"/>
-      <c r="H159" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I159" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="160">
       <c r="A160" s="9" t="n">
@@ -7062,16 +5532,6 @@
       </c>
       <c r="F160" s="10" t="n"/>
       <c r="G160" s="10" t="n"/>
-      <c r="H160" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I160" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="161">
       <c r="A161" s="9" t="n">
@@ -7099,16 +5559,6 @@
       </c>
       <c r="F161" s="10" t="n"/>
       <c r="G161" s="10" t="n"/>
-      <c r="H161" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I161" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="162">
       <c r="A162" s="9" t="n">
@@ -7136,16 +5586,6 @@
       </c>
       <c r="F162" s="10" t="n"/>
       <c r="G162" s="10" t="n"/>
-      <c r="H162" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I162" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="163">
       <c r="A163" s="9" t="n">
@@ -7173,16 +5613,6 @@
       </c>
       <c r="F163" s="10" t="n"/>
       <c r="G163" s="10" t="n"/>
-      <c r="H163" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I163" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="164">
       <c r="A164" s="9" t="n">
@@ -7210,16 +5640,6 @@
       </c>
       <c r="F164" s="10" t="n"/>
       <c r="G164" s="10" t="n"/>
-      <c r="H164" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I164" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="165">
       <c r="A165" s="9" t="n">
@@ -7247,16 +5667,6 @@
       </c>
       <c r="F165" s="10" t="n"/>
       <c r="G165" s="10" t="n"/>
-      <c r="H165" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I165" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="166">
       <c r="A166" s="9" t="n">
@@ -7284,16 +5694,6 @@
       </c>
       <c r="F166" s="10" t="n"/>
       <c r="G166" s="10" t="n"/>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I166" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="167">
       <c r="A167" s="9" t="n">
@@ -7321,16 +5721,6 @@
       </c>
       <c r="F167" s="10" t="n"/>
       <c r="G167" s="10" t="n"/>
-      <c r="H167" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I167" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="168">
       <c r="A168" s="9" t="n">
@@ -7358,16 +5748,6 @@
       </c>
       <c r="F168" s="10" t="n"/>
       <c r="G168" s="10" t="n"/>
-      <c r="H168" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I168" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="169">
       <c r="A169" s="9" t="n">
@@ -7395,16 +5775,6 @@
       </c>
       <c r="F169" s="10" t="n"/>
       <c r="G169" s="10" t="n"/>
-      <c r="H169" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I169" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="170">
       <c r="A170" s="9" t="n">
@@ -7432,16 +5802,6 @@
       </c>
       <c r="F170" s="10" t="n"/>
       <c r="G170" s="10" t="n"/>
-      <c r="H170" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I170" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="171">
       <c r="A171" s="9" t="n">
@@ -7469,16 +5829,6 @@
       </c>
       <c r="F171" s="10" t="n"/>
       <c r="G171" s="10" t="n"/>
-      <c r="H171" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I171" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="172">
       <c r="A172" s="9" t="n">
@@ -7506,16 +5856,6 @@
       </c>
       <c r="F172" s="10" t="n"/>
       <c r="G172" s="10" t="n"/>
-      <c r="H172" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I172" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="173">
       <c r="A173" s="9" t="n">
@@ -7543,16 +5883,6 @@
       </c>
       <c r="F173" s="10" t="n"/>
       <c r="G173" s="10" t="n"/>
-      <c r="H173" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I173" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="174">
       <c r="A174" s="9" t="n">
@@ -7580,16 +5910,6 @@
       </c>
       <c r="F174" s="10" t="n"/>
       <c r="G174" s="10" t="n"/>
-      <c r="H174" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I174" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="175">
       <c r="A175" s="9" t="n">
@@ -7617,16 +5937,6 @@
       </c>
       <c r="F175" s="10" t="n"/>
       <c r="G175" s="10" t="n"/>
-      <c r="H175" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="176">
       <c r="A176" s="9" t="n">
@@ -7654,16 +5964,6 @@
       </c>
       <c r="F176" s="10" t="n"/>
       <c r="G176" s="10" t="n"/>
-      <c r="H176" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I176" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="177">
       <c r="A177" s="9" t="n">
@@ -7691,16 +5991,6 @@
       </c>
       <c r="F177" s="10" t="n"/>
       <c r="G177" s="10" t="n"/>
-      <c r="H177" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I177" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="178">
       <c r="A178" s="9" t="n">
@@ -7728,16 +6018,6 @@
       </c>
       <c r="F178" s="10" t="n"/>
       <c r="G178" s="10" t="n"/>
-      <c r="H178" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="179">
       <c r="A179" s="9" t="n">
@@ -7765,16 +6045,6 @@
       </c>
       <c r="F179" s="10" t="n"/>
       <c r="G179" s="10" t="n"/>
-      <c r="H179" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I179" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="180">
       <c r="A180" s="9" t="n">
@@ -7802,16 +6072,6 @@
       </c>
       <c r="F180" s="10" t="n"/>
       <c r="G180" s="10" t="n"/>
-      <c r="H180" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I180" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="181">
       <c r="A181" s="9" t="n">
@@ -7839,16 +6099,6 @@
       </c>
       <c r="F181" s="10" t="n"/>
       <c r="G181" s="10" t="n"/>
-      <c r="H181" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I181" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="182">
       <c r="A182" s="9" t="n">
@@ -7876,16 +6126,6 @@
       </c>
       <c r="F182" s="10" t="n"/>
       <c r="G182" s="10" t="n"/>
-      <c r="H182" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I182" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="183">
       <c r="A183" s="9" t="n">
@@ -7913,16 +6153,6 @@
       </c>
       <c r="F183" s="10" t="n"/>
       <c r="G183" s="10" t="n"/>
-      <c r="H183" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I183" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="184">
       <c r="A184" s="9" t="n">
@@ -7950,16 +6180,6 @@
       </c>
       <c r="F184" s="10" t="n"/>
       <c r="G184" s="10" t="n"/>
-      <c r="H184" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I184" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="185">
       <c r="A185" s="9" t="n">
@@ -7987,16 +6207,6 @@
       </c>
       <c r="F185" s="10" t="n"/>
       <c r="G185" s="10" t="n"/>
-      <c r="H185" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I185" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="186">
       <c r="A186" s="9" t="n">
@@ -8024,16 +6234,6 @@
       </c>
       <c r="F186" s="10" t="n"/>
       <c r="G186" s="10" t="n"/>
-      <c r="H186" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I186" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="187">
       <c r="A187" s="9" t="n">
@@ -8061,16 +6261,6 @@
       </c>
       <c r="F187" s="10" t="n"/>
       <c r="G187" s="10" t="n"/>
-      <c r="H187" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I187" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="188">
       <c r="A188" s="9" t="n">
@@ -8098,16 +6288,6 @@
       </c>
       <c r="F188" s="10" t="n"/>
       <c r="G188" s="10" t="n"/>
-      <c r="H188" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I188" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="189">
       <c r="A189" s="9" t="n">
@@ -8135,16 +6315,6 @@
       </c>
       <c r="F189" s="10" t="n"/>
       <c r="G189" s="10" t="n"/>
-      <c r="H189" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I189" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="190">
       <c r="A190" s="9" t="n">
@@ -8172,16 +6342,6 @@
       </c>
       <c r="F190" s="10" t="n"/>
       <c r="G190" s="10" t="n"/>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I190" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="191">
       <c r="A191" s="9" t="n">
@@ -8209,16 +6369,6 @@
       </c>
       <c r="F191" s="10" t="n"/>
       <c r="G191" s="10" t="n"/>
-      <c r="H191" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I191" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="192">
       <c r="A192" s="9" t="n">
@@ -8246,16 +6396,6 @@
       </c>
       <c r="F192" s="10" t="n"/>
       <c r="G192" s="10" t="n"/>
-      <c r="H192" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I192" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="193">
       <c r="A193" s="9" t="n">
@@ -8283,16 +6423,6 @@
       </c>
       <c r="F193" s="10" t="n"/>
       <c r="G193" s="10" t="n"/>
-      <c r="H193" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I193" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="194">
       <c r="A194" s="9" t="n">
@@ -8320,16 +6450,6 @@
       </c>
       <c r="F194" s="10" t="n"/>
       <c r="G194" s="10" t="n"/>
-      <c r="H194" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I194" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="195">
       <c r="A195" s="9" t="n">
@@ -8357,16 +6477,6 @@
       </c>
       <c r="F195" s="10" t="n"/>
       <c r="G195" s="10" t="n"/>
-      <c r="H195" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I195" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="196">
       <c r="A196" s="9" t="n">
@@ -8394,16 +6504,6 @@
       </c>
       <c r="F196" s="10" t="n"/>
       <c r="G196" s="10" t="n"/>
-      <c r="H196" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I196" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="197">
       <c r="A197" s="9" t="n">
@@ -8431,16 +6531,6 @@
       </c>
       <c r="F197" s="10" t="n"/>
       <c r="G197" s="10" t="n"/>
-      <c r="H197" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I197" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="198">
       <c r="A198" s="9" t="n">
@@ -8468,16 +6558,6 @@
       </c>
       <c r="F198" s="10" t="n"/>
       <c r="G198" s="10" t="n"/>
-      <c r="H198" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I198" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="199">
       <c r="A199" s="9" t="n">
@@ -8505,16 +6585,6 @@
       </c>
       <c r="F199" s="10" t="n"/>
       <c r="G199" s="10" t="n"/>
-      <c r="H199" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I199" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
     <row r="200">
       <c r="A200" s="9" t="n">
@@ -8542,16 +6612,6 @@
       </c>
       <c r="F200" s="10" t="n"/>
       <c r="G200" s="10" t="n"/>
-      <c r="H200" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I200" t="inlineStr">
-        <is>
-          <t>no address, no role - awaiting transport office confirmation</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>